<commit_message>
V5: Link LLM to deterministic tools for data analysis
</commit_message>
<xml_diff>
--- a/data/sample_sales.xlsx
+++ b/data/sample_sales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,14 +429,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Revenue</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Customer_Satisfaction</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -444,52 +459,200 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1200</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>25</v>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Western Cape</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Keyboard</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>45</v>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>invalid_date</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KwaZulu-Natal</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Western Cape</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KwaZulu-Natal</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>